<commit_message>
fix(TRANS_DAYA_PRIMA): VAT 列補上費用名稱 "VAT (11%)"
VAT 列之前 Description 留空(補 N/A)，使用者提供新版正確答案
(OK_VAT.xlsx) 要求這一列要填 "VAT (11%)" 作為費用名稱，百分比直接
照抄 PDF 印的數字。同步修正 test_samples 下三份 regression fixture
的 VAT 列，重新驗證 100% 正確率。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JhL7qxuxZLsZyoRKZr1of6
</commit_message>
<xml_diff>
--- a/test_samples/TRANS_DAYA_PRIMA/sample1_ref.xlsx
+++ b/test_samples/TRANS_DAYA_PRIMA/sample1_ref.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffrey.hu\Desktop\印尼供應商帳單\已丟測試\07. PT. TRANS DAYA PRIMA____________________OK\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffrey.hu\Desktop\印尼sample\## 印尼 TOP 15 間 sample\10-TRANS DAYA PRIMA___VAT OK\$ 10-PT. TRANS DAYA PRIMA______OK VAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC531C6-D6CF-4E21-8E6F-4B8BEE2D89CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C98859-1559-454A-B144-8E1B67D86F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12420" yWindow="6480" windowWidth="21660" windowHeight="14550" tabRatio="819" xr2:uid="{B2E6A21A-966E-4572-9141-AA1879003F42}"/>
+    <workbookView xWindow="9420" yWindow="6570" windowWidth="28800" windowHeight="12855" tabRatio="819" xr2:uid="{B2E6A21A-966E-4572-9141-AA1879003F42}"/>
   </bookViews>
   <sheets>
     <sheet name="DWIHARTA" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="31">
   <si>
     <t>INVOICE DATE
 發票日期</t>
@@ -166,11 +166,11 @@
     <t>VAT</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>LCL Lokal Serang - GSI-2 40"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VAT (11%)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -209,7 +209,7 @@
       <charset val="136"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -219,6 +219,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -237,7 +243,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -257,6 +263,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="15" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -735,7 +747,7 @@
         <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3">
@@ -775,106 +787,109 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+    <row r="4" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
         <v>46048</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="8">
+        <v>7560000</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>46048</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F4">
-        <v>7560000</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" t="s">
-        <v>16</v>
-      </c>
-      <c r="K4" t="s">
-        <v>16</v>
-      </c>
-      <c r="L4" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N4" t="s">
-        <v>16</v>
-      </c>
-      <c r="O4" t="s">
-        <v>16</v>
-      </c>
-      <c r="P4" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>16</v>
-      </c>
-      <c r="R4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
-        <v>46048</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5">
+      <c r="G5" s="8">
         <v>831600</v>
       </c>
-      <c r="H5" t="s">
-        <v>16</v>
-      </c>
-      <c r="I5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" t="s">
-        <v>16</v>
-      </c>
-      <c r="K5" t="s">
-        <v>16</v>
-      </c>
-      <c r="L5" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" t="s">
-        <v>16</v>
-      </c>
-      <c r="N5" t="s">
-        <v>16</v>
-      </c>
-      <c r="O5" t="s">
-        <v>16</v>
-      </c>
-      <c r="P5" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>16</v>
-      </c>
-      <c r="R5" t="s">
+      <c r="H5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="R5" s="8" t="s">
         <v>16</v>
       </c>
     </row>
@@ -943,6 +958,9 @@
       </c>
       <c r="D7" t="s">
         <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
       </c>
       <c r="G7">
         <v>425700</v>

</xml_diff>